<commit_message>
Update Lead 231 date and dashboard Won Value column to reflect 30839768
</commit_message>
<xml_diff>
--- a/costing-report-updated-latest.xlsx
+++ b/costing-report-updated-latest.xlsx
@@ -7366,13 +7366,13 @@
         <v>316</v>
       </c>
       <c r="J161" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
       <c r="K161" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
       <c r="L161" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
     </row>
     <row r="162" spans="1:12">

</xml_diff>

<commit_message>
Update Lead 231 GA INFRA date to August and regenerate Costing September report
</commit_message>
<xml_diff>
--- a/costing-report-updated-latest.xlsx
+++ b/costing-report-updated-latest.xlsx
@@ -7366,13 +7366,13 @@
         <v>316</v>
       </c>
       <c r="J161" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="K161" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="L161" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
     </row>
     <row r="162" spans="1:12">

</xml_diff>